<commit_message>
Update task distribution document
</commit_message>
<xml_diff>
--- a/docs/Vorschlag Arbeitsteilung - erweiterte Version.xlsx
+++ b/docs/Vorschlag Arbeitsteilung - erweiterte Version.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Notebook\Documents\Mobile-Applications-SS26\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BF34D87-F32E-460D-A1D7-7744ACF05835}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11C68240-9737-4388-8AEF-B3085B965BA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{37DEA95C-12DA-4A15-A450-B2693DE4C3E5}"/>
   </bookViews>
@@ -437,9 +437,6 @@
     <t>keine externen libraries mit downloads</t>
   </si>
   <si>
-    <t>camelCase</t>
-  </si>
-  <si>
     <t>Klassennamen mit Anfangsbuchstaben gemäß Fkt. (zb I bei Interface)</t>
   </si>
   <si>
@@ -447,6 +444,9 @@
   </si>
   <si>
     <t>Package-Struktur gemäß Intellij</t>
+  </si>
+  <si>
+    <t>CamelCase</t>
   </si>
 </sst>
 </file>
@@ -1739,22 +1739,22 @@
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D104" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D105" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>